<commit_message>
Update points for 2026-04-24
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB9"/>
+  <dimension ref="A1:AC9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -523,6 +523,11 @@
           <t>2026-04-23</t>
         </is>
       </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -611,6 +616,9 @@
       <c r="AB2" t="n">
         <v>30</v>
       </c>
+      <c r="AC2" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -699,6 +707,9 @@
       <c r="AB3" t="n">
         <v>-20</v>
       </c>
+      <c r="AC3" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -787,6 +798,9 @@
       <c r="AB4" t="n">
         <v>0</v>
       </c>
+      <c r="AC4" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -875,6 +889,9 @@
       <c r="AB5" t="n">
         <v>-20</v>
       </c>
+      <c r="AC5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -963,6 +980,9 @@
       <c r="AB6" t="n">
         <v>10</v>
       </c>
+      <c r="AC6" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1051,6 +1071,9 @@
       <c r="AB7" t="n">
         <v>0</v>
       </c>
+      <c r="AC7" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1139,6 +1162,9 @@
       <c r="AB8" t="n">
         <v>0</v>
       </c>
+      <c r="AC8" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1226,6 +1252,9 @@
       </c>
       <c r="AB9" t="n">
         <v>0</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>-20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-04-25
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -525,7 +525,7 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
         <v>30</v>
       </c>
       <c r="AC2" t="n">
-        <v>60</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="3">
@@ -708,7 +708,7 @@
         <v>-20</v>
       </c>
       <c r="AC3" t="n">
-        <v>-20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         <v>0</v>
       </c>
       <c r="AC4" t="n">
-        <v>28</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="5">
@@ -890,7 +890,7 @@
         <v>-20</v>
       </c>
       <c r="AC5" t="n">
-        <v>-20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -981,7 +981,7 @@
         <v>10</v>
       </c>
       <c r="AC6" t="n">
-        <v>12</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="7">
@@ -1072,7 +1072,7 @@
         <v>0</v>
       </c>
       <c r="AC7" t="n">
-        <v>-20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Update points for 2026-04-27
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,6 +533,11 @@
           <t>2026-04-25</t>
         </is>
       </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -627,6 +632,9 @@
       <c r="AD2" t="n">
         <v>16</v>
       </c>
+      <c r="AE2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -721,6 +729,9 @@
       <c r="AD3" t="n">
         <v>-20</v>
       </c>
+      <c r="AE3" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -815,6 +826,9 @@
       <c r="AD4" t="n">
         <v>-20</v>
       </c>
+      <c r="AE4" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -909,6 +923,9 @@
       <c r="AD5" t="n">
         <v>4</v>
       </c>
+      <c r="AE5" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1003,6 +1020,9 @@
       <c r="AD6" t="n">
         <v>40</v>
       </c>
+      <c r="AE6" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1097,6 +1117,9 @@
       <c r="AD7" t="n">
         <v>0</v>
       </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1191,6 +1214,9 @@
       <c r="AD8" t="n">
         <v>0</v>
       </c>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1283,6 +1309,9 @@
         <v>4</v>
       </c>
       <c r="AD9" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE9" t="n">
         <v>-20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update points for 2026-04-28
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AF9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -538,6 +538,11 @@
           <t>2026-04-27</t>
         </is>
       </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -635,6 +640,9 @@
       <c r="AE2" t="n">
         <v>4</v>
       </c>
+      <c r="AF2" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -732,6 +740,9 @@
       <c r="AE3" t="n">
         <v>-20</v>
       </c>
+      <c r="AF3" t="n">
+        <v>-8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -829,6 +840,9 @@
       <c r="AE4" t="n">
         <v>40</v>
       </c>
+      <c r="AF4" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -926,6 +940,9 @@
       <c r="AE5" t="n">
         <v>16</v>
       </c>
+      <c r="AF5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1023,6 +1040,9 @@
       <c r="AE6" t="n">
         <v>-20</v>
       </c>
+      <c r="AF6" t="n">
+        <v>-8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1120,6 +1140,9 @@
       <c r="AE7" t="n">
         <v>0</v>
       </c>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1217,6 +1240,9 @@
       <c r="AE8" t="n">
         <v>0</v>
       </c>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1313,6 +1339,9 @@
       </c>
       <c r="AE9" t="n">
         <v>-20</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-04-29
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF9"/>
+  <dimension ref="A1:AG9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,6 +543,11 @@
           <t>2026-04-28</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -643,6 +648,9 @@
       <c r="AF2" t="n">
         <v>-20</v>
       </c>
+      <c r="AG2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -743,6 +751,9 @@
       <c r="AF3" t="n">
         <v>-8</v>
       </c>
+      <c r="AG3" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -843,6 +854,9 @@
       <c r="AF4" t="n">
         <v>40</v>
       </c>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -943,6 +957,9 @@
       <c r="AF5" t="n">
         <v>-20</v>
       </c>
+      <c r="AG5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1043,6 +1060,9 @@
       <c r="AF6" t="n">
         <v>-8</v>
       </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1143,6 +1163,9 @@
       <c r="AF7" t="n">
         <v>0</v>
       </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1243,6 +1266,9 @@
       <c r="AF8" t="n">
         <v>0</v>
       </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1342,6 +1368,9 @@
       </c>
       <c r="AF9" t="n">
         <v>16</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>-20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-04-30
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG9"/>
+  <dimension ref="A1:AH9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,6 +548,11 @@
           <t>2026-04-29</t>
         </is>
       </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -651,6 +656,9 @@
       <c r="AG2" t="n">
         <v>30</v>
       </c>
+      <c r="AH2" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -754,6 +762,9 @@
       <c r="AG3" t="n">
         <v>10</v>
       </c>
+      <c r="AH3" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -857,6 +868,9 @@
       <c r="AG4" t="n">
         <v>0</v>
       </c>
+      <c r="AH4" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -960,6 +974,9 @@
       <c r="AG5" t="n">
         <v>-20</v>
       </c>
+      <c r="AH5" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1063,6 +1080,9 @@
       <c r="AG6" t="n">
         <v>0</v>
       </c>
+      <c r="AH6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1166,6 +1186,9 @@
       <c r="AG7" t="n">
         <v>0</v>
       </c>
+      <c r="AH7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1269,6 +1292,9 @@
       <c r="AG8" t="n">
         <v>0</v>
       </c>
+      <c r="AH8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1370,6 +1396,9 @@
         <v>16</v>
       </c>
       <c r="AG9" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AH9" t="n">
         <v>-20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update points for 2026-05-01
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH9"/>
+  <dimension ref="A1:AI9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,6 +553,11 @@
           <t>2026-04-30</t>
         </is>
       </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -659,6 +664,9 @@
       <c r="AH2" t="n">
         <v>-20</v>
       </c>
+      <c r="AI2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -765,6 +773,9 @@
       <c r="AH3" t="n">
         <v>-20</v>
       </c>
+      <c r="AI3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -871,6 +882,9 @@
       <c r="AH4" t="n">
         <v>40</v>
       </c>
+      <c r="AI4" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -977,6 +991,9 @@
       <c r="AH5" t="n">
         <v>16</v>
       </c>
+      <c r="AI5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1083,6 +1100,9 @@
       <c r="AH6" t="n">
         <v>4</v>
       </c>
+      <c r="AI6" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1189,6 +1209,9 @@
       <c r="AH7" t="n">
         <v>0</v>
       </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1295,6 +1318,9 @@
       <c r="AH8" t="n">
         <v>0</v>
       </c>
+      <c r="AI8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1400,6 +1426,9 @@
       </c>
       <c r="AH9" t="n">
         <v>-20</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-05-02
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI9"/>
+  <dimension ref="A1:AJ9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,11 @@
           <t>2026-05-01</t>
         </is>
       </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -667,6 +672,9 @@
       <c r="AI2" t="n">
         <v>10</v>
       </c>
+      <c r="AJ2" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -776,6 +784,9 @@
       <c r="AI3" t="n">
         <v>0</v>
       </c>
+      <c r="AJ3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -885,6 +896,9 @@
       <c r="AI4" t="n">
         <v>30</v>
       </c>
+      <c r="AJ4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -994,6 +1008,9 @@
       <c r="AI5" t="n">
         <v>-20</v>
       </c>
+      <c r="AJ5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1103,6 +1120,9 @@
       <c r="AI6" t="n">
         <v>-20</v>
       </c>
+      <c r="AJ6" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1212,6 +1232,9 @@
       <c r="AI7" t="n">
         <v>0</v>
       </c>
+      <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1321,6 +1344,9 @@
       <c r="AI8" t="n">
         <v>0</v>
       </c>
+      <c r="AJ8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1429,6 +1455,9 @@
       </c>
       <c r="AI9" t="n">
         <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>-20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-05-04
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ9"/>
+  <dimension ref="A1:AK9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,6 +563,11 @@
           <t>2026-05-02</t>
         </is>
       </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -675,6 +680,9 @@
       <c r="AJ2" t="n">
         <v>-20</v>
       </c>
+      <c r="AK2" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -787,6 +795,9 @@
       <c r="AJ3" t="n">
         <v>16</v>
       </c>
+      <c r="AK3" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -899,6 +910,9 @@
       <c r="AJ4" t="n">
         <v>4</v>
       </c>
+      <c r="AK4" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1011,6 +1025,9 @@
       <c r="AJ5" t="n">
         <v>-20</v>
       </c>
+      <c r="AK5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1123,6 +1140,9 @@
       <c r="AJ6" t="n">
         <v>40</v>
       </c>
+      <c r="AK6" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1235,6 +1255,9 @@
       <c r="AJ7" t="n">
         <v>0</v>
       </c>
+      <c r="AK7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1347,6 +1370,9 @@
       <c r="AJ8" t="n">
         <v>0</v>
       </c>
+      <c r="AK8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1458,6 +1484,9 @@
       </c>
       <c r="AJ9" t="n">
         <v>-20</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-05-05
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK9"/>
+  <dimension ref="A1:AL9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,6 +568,11 @@
           <t>2026-05-04</t>
         </is>
       </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -683,6 +688,9 @@
       <c r="AK2" t="n">
         <v>-20</v>
       </c>
+      <c r="AL2" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -798,6 +806,9 @@
       <c r="AK3" t="n">
         <v>40</v>
       </c>
+      <c r="AL3" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -913,6 +924,9 @@
       <c r="AK4" t="n">
         <v>16</v>
       </c>
+      <c r="AL4" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1028,6 +1042,9 @@
       <c r="AK5" t="n">
         <v>-20</v>
       </c>
+      <c r="AL5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1143,6 +1160,9 @@
       <c r="AK6" t="n">
         <v>-20</v>
       </c>
+      <c r="AL6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1258,6 +1278,9 @@
       <c r="AK7" t="n">
         <v>0</v>
       </c>
+      <c r="AL7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1373,6 +1396,9 @@
       <c r="AK8" t="n">
         <v>0</v>
       </c>
+      <c r="AL8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1487,6 +1513,9 @@
       </c>
       <c r="AK9" t="n">
         <v>4</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-05-06
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL9"/>
+  <dimension ref="A1:AM9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,6 +573,11 @@
           <t>2026-05-05</t>
         </is>
       </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -691,6 +696,9 @@
       <c r="AL2" t="n">
         <v>-20</v>
       </c>
+      <c r="AM2" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -809,6 +817,9 @@
       <c r="AL3" t="n">
         <v>10</v>
       </c>
+      <c r="AM3" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -927,6 +938,9 @@
       <c r="AL4" t="n">
         <v>30</v>
       </c>
+      <c r="AM4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1045,6 +1059,9 @@
       <c r="AL5" t="n">
         <v>-20</v>
       </c>
+      <c r="AM5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1163,6 +1180,9 @@
       <c r="AL6" t="n">
         <v>0</v>
       </c>
+      <c r="AM6" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1281,6 +1301,9 @@
       <c r="AL7" t="n">
         <v>0</v>
       </c>
+      <c r="AM7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1399,6 +1422,9 @@
       <c r="AL8" t="n">
         <v>0</v>
       </c>
+      <c r="AM8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1515,6 +1541,9 @@
         <v>4</v>
       </c>
       <c r="AL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update points for 2026-05-07
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM9"/>
+  <dimension ref="A1:AN9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -578,6 +578,11 @@
           <t>2026-05-06</t>
         </is>
       </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -699,6 +704,9 @@
       <c r="AM2" t="n">
         <v>-20</v>
       </c>
+      <c r="AN2" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -820,6 +828,9 @@
       <c r="AM3" t="n">
         <v>30</v>
       </c>
+      <c r="AN3" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -941,6 +952,9 @@
       <c r="AM4" t="n">
         <v>0</v>
       </c>
+      <c r="AN4" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1062,6 +1076,9 @@
       <c r="AM5" t="n">
         <v>-20</v>
       </c>
+      <c r="AN5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1183,6 +1200,9 @@
       <c r="AM6" t="n">
         <v>10</v>
       </c>
+      <c r="AN6" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1304,6 +1324,9 @@
       <c r="AM7" t="n">
         <v>0</v>
       </c>
+      <c r="AN7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1425,6 +1448,9 @@
       <c r="AM8" t="n">
         <v>0</v>
       </c>
+      <c r="AN8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1544,6 +1570,9 @@
         <v>0</v>
       </c>
       <c r="AM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update points for 2026-05-08
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN9"/>
+  <dimension ref="A1:AO9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,6 +583,11 @@
           <t>2026-05-07</t>
         </is>
       </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -707,6 +712,9 @@
       <c r="AN2" t="n">
         <v>-20</v>
       </c>
+      <c r="AO2" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -831,6 +839,9 @@
       <c r="AN3" t="n">
         <v>30</v>
       </c>
+      <c r="AO3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -955,6 +966,9 @@
       <c r="AN4" t="n">
         <v>10</v>
       </c>
+      <c r="AO4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1079,6 +1093,9 @@
       <c r="AN5" t="n">
         <v>0</v>
       </c>
+      <c r="AO5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1203,6 +1220,9 @@
       <c r="AN6" t="n">
         <v>-20</v>
       </c>
+      <c r="AO6" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1327,6 +1347,9 @@
       <c r="AN7" t="n">
         <v>0</v>
       </c>
+      <c r="AO7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1451,6 +1474,9 @@
       <c r="AN8" t="n">
         <v>0</v>
       </c>
+      <c r="AO8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1574,6 +1600,9 @@
       </c>
       <c r="AN9" t="n">
         <v>0</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>-20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-05-10
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO9"/>
+  <dimension ref="A1:AP9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -588,6 +588,11 @@
           <t>2026-05-08</t>
         </is>
       </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -715,6 +720,9 @@
       <c r="AO2" t="n">
         <v>-20</v>
       </c>
+      <c r="AP2" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -842,6 +850,9 @@
       <c r="AO3" t="n">
         <v>16</v>
       </c>
+      <c r="AP3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -969,6 +980,9 @@
       <c r="AO4" t="n">
         <v>4</v>
       </c>
+      <c r="AP4" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1096,6 +1110,9 @@
       <c r="AO5" t="n">
         <v>-20</v>
       </c>
+      <c r="AP5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1223,6 +1240,9 @@
       <c r="AO6" t="n">
         <v>40</v>
       </c>
+      <c r="AP6" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1350,6 +1370,9 @@
       <c r="AO7" t="n">
         <v>0</v>
       </c>
+      <c r="AP7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1477,6 +1500,9 @@
       <c r="AO8" t="n">
         <v>0</v>
       </c>
+      <c r="AP8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1603,6 +1629,9 @@
       </c>
       <c r="AO9" t="n">
         <v>-20</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-05-11
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ9"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -598,6 +598,11 @@
           <t>2026-05-10</t>
         </is>
       </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -731,6 +736,9 @@
       <c r="AQ2" t="n">
         <v>16</v>
       </c>
+      <c r="AR2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -864,6 +872,9 @@
       <c r="AQ3" t="n">
         <v>40</v>
       </c>
+      <c r="AR3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -997,6 +1008,9 @@
       <c r="AQ4" t="n">
         <v>-20</v>
       </c>
+      <c r="AR4" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1130,6 +1144,9 @@
       <c r="AQ5" t="n">
         <v>-20</v>
       </c>
+      <c r="AR5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1263,6 +1280,9 @@
       <c r="AQ6" t="n">
         <v>4</v>
       </c>
+      <c r="AR6" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1396,6 +1416,9 @@
       <c r="AQ7" t="n">
         <v>0</v>
       </c>
+      <c r="AR7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1529,6 +1552,9 @@
       <c r="AQ8" t="n">
         <v>0</v>
       </c>
+      <c r="AR8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1661,6 +1687,9 @@
       </c>
       <c r="AQ9" t="n">
         <v>-20</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-05-13
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AS9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -603,6 +603,11 @@
           <t>2026-05-11</t>
         </is>
       </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -739,6 +744,9 @@
       <c r="AR2" t="n">
         <v>10</v>
       </c>
+      <c r="AS2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -875,6 +883,9 @@
       <c r="AR3" t="n">
         <v>0</v>
       </c>
+      <c r="AS3" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1011,6 +1022,9 @@
       <c r="AR4" t="n">
         <v>-20</v>
       </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1147,6 +1161,9 @@
       <c r="AR5" t="n">
         <v>-20</v>
       </c>
+      <c r="AS5" t="n">
+        <v>-20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1283,6 +1300,9 @@
       <c r="AR6" t="n">
         <v>30</v>
       </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1419,6 +1439,9 @@
       <c r="AR7" t="n">
         <v>0</v>
       </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1555,6 +1578,9 @@
       <c r="AR8" t="n">
         <v>0</v>
       </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1690,6 +1716,9 @@
       </c>
       <c r="AR9" t="n">
         <v>0</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update points for 2026-05-31
</commit_message>
<xml_diff>
--- a/TeamRankApp.xlsx
+++ b/TeamRankApp.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS9"/>
+  <dimension ref="A1:AT9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,6 +608,11 @@
           <t>2026-05-13</t>
         </is>
       </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -747,6 +752,9 @@
       <c r="AS2" t="n">
         <v>30</v>
       </c>
+      <c r="AT2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -886,6 +894,9 @@
       <c r="AS3" t="n">
         <v>-20</v>
       </c>
+      <c r="AT3" t="n">
+        <v>-50</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1025,6 +1036,9 @@
       <c r="AS4" t="n">
         <v>0</v>
       </c>
+      <c r="AT4" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1164,6 +1178,9 @@
       <c r="AS5" t="n">
         <v>-20</v>
       </c>
+      <c r="AT5" t="n">
+        <v>-50</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1303,6 +1320,9 @@
       <c r="AS6" t="n">
         <v>0</v>
       </c>
+      <c r="AT6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1442,6 +1462,9 @@
       <c r="AS7" t="n">
         <v>0</v>
       </c>
+      <c r="AT7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1581,6 +1604,9 @@
       <c r="AS8" t="n">
         <v>0</v>
       </c>
+      <c r="AT8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1719,6 +1745,9 @@
       </c>
       <c r="AS9" t="n">
         <v>10</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>